<commit_message>
Logiciel de Assurance Automobile avec gestion de flotte mono complête et gestion de flotte complexe. intégration de API ASAC à. niveau de développement: 70% v4
</commit_message>
<xml_diff>
--- a/modele_import_asac.xlsx
+++ b/modele_import_asac.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,6 +652,120 @@
       </c>
       <c r="M4" t="n">
         <v>145000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LT-004-DE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Nissan</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Patrol</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>VF4MNOP901234</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Professionnel</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="L5" t="n">
+        <v>42000000</v>
+      </c>
+      <c r="M5" t="n">
+        <v>185000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LT-005-EF</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Porter</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>VF5QRST567890</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>VU</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Professionnel</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="L6" t="n">
+        <v>19000000</v>
+      </c>
+      <c r="M6" t="n">
+        <v>95000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>